<commit_message>
Sort files in supplementary folder
</commit_message>
<xml_diff>
--- a/1.Training_model/supplementary/Data Tabulation - Flowchart.xlsx
+++ b/1.Training_model/supplementary/Data Tabulation - Flowchart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\supplementary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\1.Training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C177ABD-7CF8-4571-93F1-94E5AF7E7F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="717" firstSheet="3" activeTab="10" xr2:uid="{E471D6E3-533D-4285-ABDC-6FF3DFDEE99D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="717" firstSheet="2" activeTab="2" xr2:uid="{E471D6E3-533D-4285-ABDC-6FF3DFDEE99D}"/>
   </bookViews>
   <sheets>
     <sheet name="Obs-flowchart" sheetId="19" state="hidden" r:id="rId1"/>

</xml_diff>